<commit_message>
addition of practical task dependancy diagram
</commit_message>
<xml_diff>
--- a/hardware/components and parts/Component Selection Excel.xlsx
+++ b/hardware/components and parts/Component Selection Excel.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="30131"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="30326"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://essexuniversity-my.sharepoint.com/personal/br24151_essex_ac_uk/Documents/UNI documents/Year 3/CE301/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\bendr\Documents\info and files\UNI documents\Year 3\CE301\CE301 repository\hardware\components and parts\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="77" documentId="11_F25DC773A252ABDACC104860911A7AB85ADE58ED" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{8A40031B-4639-4486-9352-5CA12205E6F4}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{46CE2DAD-0457-47A8-81AB-D08A1C0CCBDD}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="19095" yWindow="0" windowWidth="19410" windowHeight="20985" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-105" yWindow="0" windowWidth="19410" windowHeight="20985" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -105,17 +105,16 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="8">
+  <cellXfs count="7">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment horizontal="left"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="right"/>
@@ -124,7 +123,7 @@
       <alignment horizontal="left" vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
-      <alignment horizontal="left"/>
+      <alignment horizontal="center" vertical="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -406,286 +405,232 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="C4:J39"/>
+  <dimension ref="C7:K39"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <sheetData>
-    <row r="4" spans="3:10" x14ac:dyDescent="0.25">
-      <c r="F4" s="2" t="s">
+    <row r="7" spans="3:10" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="C7" s="1"/>
+    </row>
+    <row r="8" spans="3:10" x14ac:dyDescent="0.25">
+      <c r="C8" s="1"/>
+    </row>
+    <row r="9" spans="3:10" x14ac:dyDescent="0.25">
+      <c r="C9" s="1"/>
+    </row>
+    <row r="10" spans="3:10" x14ac:dyDescent="0.25">
+      <c r="C10" s="1"/>
+    </row>
+    <row r="11" spans="3:10" x14ac:dyDescent="0.25">
+      <c r="C11" s="1"/>
+    </row>
+    <row r="13" spans="3:10" x14ac:dyDescent="0.25">
+      <c r="F13" s="6" t="s">
         <v>0</v>
       </c>
-      <c r="G4" s="2"/>
-      <c r="H4" s="2"/>
-      <c r="I4" s="2"/>
-      <c r="J4" s="2"/>
-    </row>
-    <row r="5" spans="3:10" x14ac:dyDescent="0.25">
-      <c r="F5" s="2"/>
-      <c r="G5" s="2"/>
-      <c r="H5" s="2"/>
-      <c r="I5" s="2"/>
-      <c r="J5" s="2"/>
-    </row>
-    <row r="6" spans="3:10" x14ac:dyDescent="0.25">
-      <c r="D6" s="1"/>
-      <c r="E6" s="1"/>
-      <c r="F6" s="2"/>
-      <c r="G6" s="2"/>
-      <c r="H6" s="2"/>
-      <c r="I6" s="2"/>
-      <c r="J6" s="2"/>
-    </row>
-    <row r="7" spans="3:10" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="C7" s="3"/>
-      <c r="D7" s="2" t="s">
+      <c r="G13" s="6"/>
+      <c r="H13" s="6"/>
+      <c r="I13" s="6"/>
+      <c r="J13" s="6"/>
+    </row>
+    <row r="14" spans="3:10" x14ac:dyDescent="0.25">
+      <c r="F14" s="6"/>
+      <c r="G14" s="6"/>
+      <c r="H14" s="6"/>
+      <c r="I14" s="6"/>
+      <c r="J14" s="6"/>
+    </row>
+    <row r="15" spans="3:10" x14ac:dyDescent="0.25">
+      <c r="F15" s="6"/>
+      <c r="G15" s="6"/>
+      <c r="H15" s="6"/>
+      <c r="I15" s="6"/>
+      <c r="J15" s="6"/>
+    </row>
+    <row r="16" spans="3:10" x14ac:dyDescent="0.25">
+      <c r="D16" s="6" t="s">
         <v>2</v>
       </c>
-      <c r="E7" s="2"/>
-      <c r="F7" s="6" t="s">
+      <c r="E16" s="6"/>
+      <c r="F16" s="5" t="s">
         <v>4</v>
       </c>
-      <c r="G7" s="6"/>
-      <c r="H7" s="6"/>
-      <c r="I7" s="6"/>
-      <c r="J7" s="6"/>
-    </row>
-    <row r="8" spans="3:10" x14ac:dyDescent="0.25">
-      <c r="C8" s="3"/>
-      <c r="D8" s="2"/>
-      <c r="E8" s="2"/>
-      <c r="F8" s="6"/>
-      <c r="G8" s="6"/>
-      <c r="H8" s="6"/>
-      <c r="I8" s="6"/>
-      <c r="J8" s="6"/>
-    </row>
-    <row r="9" spans="3:10" x14ac:dyDescent="0.25">
-      <c r="C9" s="3"/>
-      <c r="D9" s="2"/>
-      <c r="E9" s="2"/>
-      <c r="F9" s="6"/>
-      <c r="G9" s="6"/>
-      <c r="H9" s="6"/>
-      <c r="I9" s="6"/>
-      <c r="J9" s="6"/>
-    </row>
-    <row r="10" spans="3:10" x14ac:dyDescent="0.25">
-      <c r="C10" s="3"/>
-      <c r="D10" s="2"/>
-      <c r="E10" s="2"/>
-      <c r="F10" s="6"/>
-      <c r="G10" s="6"/>
-      <c r="H10" s="6"/>
-      <c r="I10" s="6"/>
-      <c r="J10" s="6"/>
-    </row>
-    <row r="11" spans="3:10" x14ac:dyDescent="0.25">
-      <c r="C11" s="3"/>
-      <c r="D11" s="2"/>
-      <c r="E11" s="2"/>
-      <c r="F11" s="6"/>
-      <c r="G11" s="6"/>
-      <c r="H11" s="6"/>
-      <c r="I11" s="6"/>
-      <c r="J11" s="6"/>
-    </row>
-    <row r="12" spans="3:10" x14ac:dyDescent="0.25">
-      <c r="D12" s="2"/>
-      <c r="E12" s="2"/>
-      <c r="F12" s="6"/>
-      <c r="G12" s="6"/>
-      <c r="H12" s="6"/>
-      <c r="I12" s="6"/>
-      <c r="J12" s="6"/>
-    </row>
-    <row r="13" spans="3:10" x14ac:dyDescent="0.25">
-      <c r="D13" s="2"/>
-      <c r="E13" s="2"/>
-      <c r="F13" s="5" t="s">
+      <c r="G16" s="5"/>
+      <c r="H16" s="5"/>
+      <c r="I16" s="5"/>
+      <c r="J16" s="5"/>
+    </row>
+    <row r="17" spans="4:11" x14ac:dyDescent="0.25">
+      <c r="D17" s="6"/>
+      <c r="E17" s="6"/>
+      <c r="F17" s="5"/>
+      <c r="G17" s="5"/>
+      <c r="H17" s="5"/>
+      <c r="I17" s="5"/>
+      <c r="J17" s="5"/>
+    </row>
+    <row r="18" spans="4:11" x14ac:dyDescent="0.25">
+      <c r="D18" s="6"/>
+      <c r="E18" s="6"/>
+      <c r="F18" s="5"/>
+      <c r="G18" s="5"/>
+      <c r="H18" s="5"/>
+      <c r="I18" s="5"/>
+      <c r="J18" s="5"/>
+    </row>
+    <row r="19" spans="4:11" x14ac:dyDescent="0.25">
+      <c r="D19" s="6"/>
+      <c r="E19" s="6"/>
+      <c r="F19" s="5"/>
+      <c r="G19" s="5"/>
+      <c r="H19" s="5"/>
+      <c r="I19" s="5"/>
+      <c r="J19" s="5"/>
+    </row>
+    <row r="20" spans="4:11" x14ac:dyDescent="0.25">
+      <c r="D20" s="6"/>
+      <c r="E20" s="6"/>
+      <c r="F20" s="5"/>
+      <c r="G20" s="5"/>
+      <c r="H20" s="5"/>
+      <c r="I20" s="5"/>
+      <c r="J20" s="5"/>
+    </row>
+    <row r="21" spans="4:11" x14ac:dyDescent="0.25">
+      <c r="D21" s="6"/>
+      <c r="E21" s="6"/>
+      <c r="F21" s="5"/>
+      <c r="G21" s="5"/>
+      <c r="H21" s="5"/>
+      <c r="I21" s="5"/>
+      <c r="J21" s="5"/>
+    </row>
+    <row r="22" spans="4:11" x14ac:dyDescent="0.25">
+      <c r="D22" s="6"/>
+      <c r="E22" s="6"/>
+      <c r="F22" s="4" t="s">
         <v>3</v>
       </c>
-      <c r="G13" s="5"/>
-      <c r="H13" s="5"/>
-      <c r="I13" s="5"/>
-      <c r="J13" s="7">
-        <v>24</v>
-      </c>
-    </row>
-    <row r="14" spans="3:10" x14ac:dyDescent="0.25">
-      <c r="F14" s="4"/>
-      <c r="G14" s="4"/>
-      <c r="H14" s="4"/>
-      <c r="I14" s="4"/>
-      <c r="J14" s="4"/>
-    </row>
-    <row r="15" spans="3:10" x14ac:dyDescent="0.25">
-      <c r="F15" s="4"/>
-      <c r="G15" s="4"/>
-      <c r="H15" s="4"/>
-      <c r="I15" s="4"/>
-      <c r="J15" s="4"/>
-    </row>
-    <row r="16" spans="3:10" x14ac:dyDescent="0.25">
-      <c r="F16" s="4"/>
-      <c r="G16" s="4"/>
-      <c r="H16" s="4"/>
-      <c r="I16" s="4"/>
-      <c r="J16" s="4"/>
-    </row>
-    <row r="17" spans="6:10" x14ac:dyDescent="0.25">
-      <c r="F17" s="4"/>
-      <c r="G17" s="4"/>
-      <c r="H17" s="4"/>
-      <c r="I17" s="4"/>
-      <c r="J17" s="4"/>
-    </row>
-    <row r="18" spans="6:10" x14ac:dyDescent="0.25">
-      <c r="F18" s="4"/>
-      <c r="G18" s="4"/>
-      <c r="H18" s="4"/>
-      <c r="I18" s="4"/>
-      <c r="J18" s="4"/>
-    </row>
-    <row r="19" spans="6:10" x14ac:dyDescent="0.25">
-      <c r="F19" s="4"/>
-      <c r="G19" s="4"/>
-      <c r="H19" s="4"/>
-      <c r="I19" s="4"/>
-      <c r="J19" s="4"/>
-    </row>
-    <row r="20" spans="6:10" x14ac:dyDescent="0.25">
-      <c r="F20" s="4"/>
-      <c r="G20" s="4"/>
-      <c r="H20" s="4"/>
-      <c r="I20" s="4"/>
-      <c r="J20" s="4"/>
-    </row>
-    <row r="21" spans="6:10" x14ac:dyDescent="0.25">
-      <c r="F21" s="4"/>
-      <c r="G21" s="4"/>
-      <c r="H21" s="4"/>
-      <c r="I21" s="4"/>
-      <c r="J21" s="4"/>
-    </row>
-    <row r="22" spans="6:10" x14ac:dyDescent="0.25">
-      <c r="F22" s="4"/>
       <c r="G22" s="4"/>
       <c r="H22" s="4"/>
       <c r="I22" s="4"/>
       <c r="J22" s="4"/>
-    </row>
-    <row r="23" spans="6:10" x14ac:dyDescent="0.25">
-      <c r="F23" s="4"/>
-      <c r="G23" s="4"/>
-      <c r="H23" s="4"/>
-      <c r="I23" s="4"/>
-      <c r="J23" s="4"/>
-    </row>
-    <row r="24" spans="6:10" x14ac:dyDescent="0.25">
-      <c r="F24" s="4"/>
-      <c r="G24" s="4"/>
-      <c r="H24" s="4"/>
-      <c r="I24" s="4"/>
-      <c r="J24" s="4"/>
-    </row>
-    <row r="25" spans="6:10" x14ac:dyDescent="0.25">
-      <c r="F25" s="4"/>
-      <c r="G25" s="4"/>
-      <c r="H25" s="4"/>
-      <c r="I25" s="4"/>
-      <c r="J25" s="4"/>
-    </row>
-    <row r="26" spans="6:10" x14ac:dyDescent="0.25">
-      <c r="F26" s="4"/>
-      <c r="G26" s="4"/>
-      <c r="H26" s="4"/>
-      <c r="I26" s="4"/>
-      <c r="J26" s="4"/>
-    </row>
-    <row r="27" spans="6:10" x14ac:dyDescent="0.25">
-      <c r="F27" s="4"/>
-      <c r="G27" s="4"/>
-      <c r="H27" s="4"/>
-      <c r="I27" s="4"/>
-      <c r="J27" s="4"/>
-    </row>
-    <row r="28" spans="6:10" x14ac:dyDescent="0.25">
-      <c r="F28" s="4"/>
-      <c r="G28" s="4"/>
-      <c r="H28" s="4"/>
-      <c r="I28" s="4"/>
-      <c r="J28" s="4"/>
-    </row>
-    <row r="29" spans="6:10" x14ac:dyDescent="0.25">
-      <c r="F29" s="4"/>
-      <c r="G29" s="4"/>
-      <c r="H29" s="4"/>
-      <c r="I29" s="4"/>
-      <c r="J29" s="4"/>
-    </row>
-    <row r="30" spans="6:10" x14ac:dyDescent="0.25">
-      <c r="F30" s="4"/>
-      <c r="G30" s="4"/>
-      <c r="H30" s="4"/>
-      <c r="I30" s="4"/>
-      <c r="J30" s="4"/>
-    </row>
-    <row r="31" spans="6:10" x14ac:dyDescent="0.25">
-      <c r="F31" s="4"/>
-      <c r="G31" s="4"/>
-      <c r="H31" s="4"/>
-      <c r="I31" s="4"/>
-      <c r="J31" s="4"/>
-    </row>
-    <row r="32" spans="6:10" x14ac:dyDescent="0.25">
-      <c r="F32" s="4"/>
-      <c r="G32" s="4"/>
-      <c r="H32" s="4"/>
-      <c r="I32" s="4"/>
-      <c r="J32" s="4"/>
+      <c r="K22" s="3">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="23" spans="4:11" x14ac:dyDescent="0.25">
+      <c r="F23" s="2"/>
+      <c r="G23" s="2"/>
+      <c r="H23" s="2"/>
+      <c r="I23" s="2"/>
+      <c r="J23" s="2"/>
+    </row>
+    <row r="24" spans="4:11" x14ac:dyDescent="0.25">
+      <c r="F24" s="2"/>
+      <c r="G24" s="2"/>
+      <c r="H24" s="2"/>
+      <c r="I24" s="2"/>
+      <c r="J24" s="2"/>
+    </row>
+    <row r="25" spans="4:11" x14ac:dyDescent="0.25">
+      <c r="F25" s="2"/>
+      <c r="G25" s="2"/>
+      <c r="H25" s="2"/>
+      <c r="I25" s="2"/>
+      <c r="J25" s="2"/>
+    </row>
+    <row r="26" spans="4:11" x14ac:dyDescent="0.25">
+      <c r="F26" s="2"/>
+      <c r="G26" s="2"/>
+      <c r="H26" s="2"/>
+      <c r="I26" s="2"/>
+      <c r="J26" s="2"/>
+    </row>
+    <row r="27" spans="4:11" x14ac:dyDescent="0.25">
+      <c r="F27" s="2"/>
+      <c r="G27" s="2"/>
+      <c r="H27" s="2"/>
+      <c r="I27" s="2"/>
+      <c r="J27" s="2"/>
+    </row>
+    <row r="28" spans="4:11" x14ac:dyDescent="0.25">
+      <c r="F28" s="2"/>
+      <c r="G28" s="2"/>
+      <c r="H28" s="2"/>
+      <c r="I28" s="2"/>
+      <c r="J28" s="2"/>
+    </row>
+    <row r="29" spans="4:11" x14ac:dyDescent="0.25">
+      <c r="F29" s="2"/>
+      <c r="G29" s="2"/>
+      <c r="H29" s="2"/>
+      <c r="I29" s="2"/>
+      <c r="J29" s="2"/>
+    </row>
+    <row r="30" spans="4:11" x14ac:dyDescent="0.25">
+      <c r="F30" s="2"/>
+      <c r="G30" s="2"/>
+      <c r="H30" s="2"/>
+      <c r="I30" s="2"/>
+      <c r="J30" s="2"/>
+    </row>
+    <row r="31" spans="4:11" x14ac:dyDescent="0.25">
+      <c r="F31" s="2"/>
+      <c r="G31" s="2"/>
+      <c r="H31" s="2"/>
+      <c r="I31" s="2"/>
+      <c r="J31" s="2"/>
+    </row>
+    <row r="32" spans="4:11" x14ac:dyDescent="0.25">
+      <c r="F32" s="2"/>
+      <c r="G32" s="2"/>
+      <c r="H32" s="2"/>
+      <c r="I32" s="2"/>
+      <c r="J32" s="2"/>
     </row>
     <row r="33" spans="6:10" x14ac:dyDescent="0.25">
-      <c r="F33" s="4"/>
-      <c r="G33" s="4"/>
-      <c r="H33" s="4"/>
-      <c r="I33" s="4"/>
-      <c r="J33" s="4"/>
+      <c r="F33" s="2"/>
+      <c r="G33" s="2"/>
+      <c r="H33" s="2"/>
+      <c r="I33" s="2"/>
+      <c r="J33" s="2"/>
     </row>
     <row r="34" spans="6:10" x14ac:dyDescent="0.25">
-      <c r="F34" s="4"/>
-      <c r="G34" s="4"/>
-      <c r="H34" s="4"/>
-      <c r="I34" s="4"/>
-      <c r="J34" s="4"/>
+      <c r="F34" s="2"/>
+      <c r="G34" s="2"/>
+      <c r="H34" s="2"/>
+      <c r="I34" s="2"/>
+      <c r="J34" s="2"/>
     </row>
     <row r="35" spans="6:10" x14ac:dyDescent="0.25">
-      <c r="F35" s="4"/>
-      <c r="G35" s="4"/>
-      <c r="H35" s="4"/>
-      <c r="I35" s="4"/>
-      <c r="J35" s="4"/>
+      <c r="F35" s="2"/>
+      <c r="G35" s="2"/>
+      <c r="H35" s="2"/>
+      <c r="I35" s="2"/>
+      <c r="J35" s="2"/>
     </row>
     <row r="36" spans="6:10" x14ac:dyDescent="0.25">
-      <c r="F36" s="4"/>
-      <c r="G36" s="4"/>
-      <c r="H36" s="4"/>
-      <c r="I36" s="4"/>
-      <c r="J36" s="4"/>
+      <c r="F36" s="2"/>
+      <c r="G36" s="2"/>
+      <c r="H36" s="2"/>
+      <c r="I36" s="2"/>
+      <c r="J36" s="2"/>
     </row>
     <row r="39" spans="6:10" x14ac:dyDescent="0.25">
-      <c r="F39" s="5" t="s">
+      <c r="F39" s="4" t="s">
         <v>1</v>
       </c>
-      <c r="G39" s="5"/>
-      <c r="H39" s="5"/>
-      <c r="I39" s="5"/>
+      <c r="G39" s="4"/>
+      <c r="H39" s="4"/>
+      <c r="I39" s="4"/>
     </row>
   </sheetData>
   <mergeCells count="5">
     <mergeCell ref="F39:I39"/>
-    <mergeCell ref="F13:I13"/>
-    <mergeCell ref="F7:J12"/>
-    <mergeCell ref="D7:E13"/>
-    <mergeCell ref="F4:J6"/>
+    <mergeCell ref="F16:J21"/>
+    <mergeCell ref="D16:E22"/>
+    <mergeCell ref="F13:J15"/>
+    <mergeCell ref="F22:J22"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>